<commit_message>
production ready static with map
</commit_message>
<xml_diff>
--- a/VRPExample/heuristicapproach/src/furgoni_con_prova.xlsx
+++ b/VRPExample/heuristicapproach/src/furgoni_con_prova.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\OQI_Project\Full Optimizer\VRPExample\heuristicapproach\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D79FEDA-36DF-4D8B-B265-C433B1754D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEBC6744-36B9-4F26-A634-38571D66B9E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="3765" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONSEGNE" sheetId="1" r:id="rId1"/>
@@ -1530,18 +1530,18 @@
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.28515625" customWidth="1"/>
+    <col min="3" max="3" width="36.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" style="10" customWidth="1"/>
     <col min="5" max="5" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.85546875" style="44" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="44" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
     <col min="9" max="9" width="27.42578125" style="45" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.42578125" style="45" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="27.42578125" style="50" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23" style="50" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.85546875" style="50" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" style="50" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" style="10" customWidth="1"/>
     <col min="14" max="14" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="18.42578125" style="10" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.85546875" style="54" bestFit="1" customWidth="1"/>
@@ -1646,7 +1646,7 @@
         <v>126</v>
       </c>
       <c r="K2" s="47">
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="L2" s="47">
         <v>0.99930555555555556</v>
@@ -1775,7 +1775,7 @@
         <v>0.25</v>
       </c>
       <c r="L4" s="47">
-        <v>0.33333333333333331</v>
+        <v>0.99930555555555556</v>
       </c>
       <c r="M4" s="35">
         <v>30</v>
@@ -2218,7 +2218,7 @@
         <v>0.75</v>
       </c>
       <c r="M11" s="35">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N11" s="34" t="s">
         <v>108</v>
@@ -2276,7 +2276,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="L12" s="47">
-        <v>0.99930555555555556</v>
+        <v>0.75</v>
       </c>
       <c r="M12" s="35">
         <v>30</v>
@@ -2339,10 +2339,10 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="L13" s="47">
-        <v>0.99930555555555556</v>
+        <v>0.75</v>
       </c>
       <c r="M13" s="35">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N13" s="34" t="s">
         <v>108</v>
@@ -2463,7 +2463,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="L15" s="47">
-        <v>0.99930555555555556</v>
+        <v>0.75</v>
       </c>
       <c r="M15" s="35">
         <v>30</v>
@@ -2472,7 +2472,7 @@
         <v>110</v>
       </c>
       <c r="O15" s="35">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="P15" s="52">
         <v>1.5</v>
@@ -2837,7 +2837,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="L21" s="47">
-        <v>0.35416666666666669</v>
+        <v>0.77083333333333337</v>
       </c>
       <c r="M21" s="35">
         <v>30</v>
@@ -2897,7 +2897,7 @@
         <v>126</v>
       </c>
       <c r="K22" s="47">
-        <v>0.33333333333333331</v>
+        <v>0.20833333333333334</v>
       </c>
       <c r="L22" s="47">
         <v>0.75</v>
@@ -3331,7 +3331,7 @@
         <v>126</v>
       </c>
       <c r="K29" s="48">
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="L29" s="48">
         <v>0.99930555555555556</v>
@@ -3827,7 +3827,7 @@
         <v>126</v>
       </c>
       <c r="K37" s="47">
-        <v>0.25</v>
+        <v>0.20833333333333334</v>
       </c>
       <c r="L37" s="47">
         <v>0.75</v>
@@ -4447,7 +4447,7 @@
         <v>126</v>
       </c>
       <c r="K47" s="47">
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="L47" s="47">
         <v>0.99930555555555556</v>

</xml_diff>